<commit_message>
Resolved data split issue (train/test)
</commit_message>
<xml_diff>
--- a/data/02_portfolio_optimization_backtest.xlsx
+++ b/data/02_portfolio_optimization_backtest.xlsx
@@ -448,13 +448,13 @@
         <v>44957</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01327584140617164</v>
+        <v>-0.0143223005375106</v>
       </c>
       <c r="C2" t="n">
         <v>10</v>
       </c>
       <c r="D2" t="n">
-        <v>0.01327584140617155</v>
+        <v>-0.0143223005375106</v>
       </c>
     </row>
     <row r="3">
@@ -462,13 +462,13 @@
         <v>44985</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.007811532004062349</v>
+        <v>0.01759315770546228</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>0.005360604742083996</v>
+        <v>0.003018882675890122</v>
       </c>
     </row>
     <row r="4">
@@ -476,13 +476,13 @@
         <v>45016</v>
       </c>
       <c r="B4" t="n">
-        <v>9.650945197502148e-06</v>
+        <v>9.642576345149367e-06</v>
       </c>
       <c r="C4" t="n">
         <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>0.005370307422184029</v>
+        <v>0.00302855436204208</v>
       </c>
     </row>
     <row r="5">
@@ -490,13 +490,13 @@
         <v>45046</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.03159173821935352</v>
+        <v>-0.02840761119052029</v>
       </c>
       <c r="C5" t="n">
         <v>10</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.02639108814340863</v>
+        <v>-0.02546509082326442</v>
       </c>
     </row>
     <row r="6">
@@ -504,13 +504,13 @@
         <v>45077</v>
       </c>
       <c r="B6" t="n">
-        <v>0.05360188891873661</v>
+        <v>0.0138504850058213</v>
       </c>
       <c r="C6" t="n">
         <v>10</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02579618860022048</v>
+        <v>-0.01196730967606274</v>
       </c>
     </row>
     <row r="7">
@@ -518,13 +518,13 @@
         <v>45107</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.0005059612217292618</v>
+        <v>-0.006580249463349672</v>
       </c>
       <c r="C7" t="n">
         <v>10</v>
       </c>
       <c r="D7" t="n">
-        <v>0.02527717550739106</v>
+        <v>-0.01846881125633881</v>
       </c>
     </row>
     <row r="8">
@@ -532,13 +532,13 @@
         <v>45138</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.01441718927685273</v>
+        <v>-0.01107544251413588</v>
       </c>
       <c r="C8" t="n">
         <v>10</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01049556040686395</v>
+        <v>-0.02933970351310067</v>
       </c>
     </row>
     <row r="9">
@@ -546,13 +546,13 @@
         <v>45169</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.01777729036170989</v>
+        <v>-0.01777727761230753</v>
       </c>
       <c r="C9" t="n">
         <v>10</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.007468312579707703</v>
+        <v>-0.04659540107099303</v>
       </c>
     </row>
     <row r="10">
@@ -560,13 +560,13 @@
         <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>0.004491610576988268</v>
+        <v>0.001572329559243646</v>
       </c>
       <c r="C10" t="n">
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.003010246754494683</v>
+        <v>-0.04509633483817821</v>
       </c>
     </row>
     <row r="11">
@@ -574,13 +574,13 @@
         <v>45230</v>
       </c>
       <c r="B11" t="n">
-        <v>0.03907173562954228</v>
+        <v>0.03907176541251828</v>
       </c>
       <c r="C11" t="n">
         <v>10</v>
       </c>
       <c r="D11" t="n">
-        <v>0.03594387330967619</v>
+        <v>-0.00778656284142154</v>
       </c>
     </row>
     <row r="12">
@@ -588,13 +588,13 @@
         <v>45260</v>
       </c>
       <c r="B12" t="n">
-        <v>0.025319759910151</v>
+        <v>0.01324342021713043</v>
       </c>
       <c r="C12" t="n">
         <v>10</v>
       </c>
       <c r="D12" t="n">
-        <v>0.06217372346226901</v>
+        <v>0.005353736651952934</v>
       </c>
     </row>
     <row r="13">
@@ -602,13 +602,13 @@
         <v>45291</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.02513223480897647</v>
+        <v>-0.03629742036736827</v>
       </c>
       <c r="C13" t="n">
         <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>0.03547892403629049</v>
+        <v>-0.03113801054520748</v>
       </c>
     </row>
     <row r="14">
@@ -616,13 +616,13 @@
         <v>45322</v>
       </c>
       <c r="B14" t="n">
-        <v>-0.0308767377645388</v>
+        <v>-0.0285878551922281</v>
       </c>
       <c r="C14" t="n">
         <v>10</v>
       </c>
       <c r="D14" t="n">
-        <v>0.003506712838115211</v>
+        <v>-0.0588356968009951</v>
       </c>
     </row>
     <row r="15">
@@ -630,13 +630,13 @@
         <v>45351</v>
       </c>
       <c r="B15" t="n">
-        <v>0.05501209632906345</v>
+        <v>0.05362457887198531</v>
       </c>
       <c r="C15" t="n">
         <v>10</v>
       </c>
       <c r="D15" t="n">
-        <v>0.05871172079162745</v>
+        <v>-0.008366157392602935</v>
       </c>
     </row>
     <row r="16">
@@ -644,13 +644,13 @@
         <v>45382</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.04502231949049337</v>
+        <v>-0.005100952935510233</v>
       </c>
       <c r="C16" t="n">
         <v>10</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01104606344981685</v>
+        <v>-0.0134244349530025</v>
       </c>
     </row>
     <row r="17">
@@ -658,13 +658,13 @@
         <v>45412</v>
       </c>
       <c r="B17" t="n">
-        <v>0.01505408354698202</v>
+        <v>0.01418645548354154</v>
       </c>
       <c r="C17" t="n">
         <v>10</v>
       </c>
       <c r="D17" t="n">
-        <v>0.02626643535883777</v>
+        <v>0.0005715753816866176</v>
       </c>
     </row>
     <row r="18">
@@ -672,13 +672,13 @@
         <v>45443</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.00557296232942169</v>
+        <v>0.009183731259777062</v>
       </c>
       <c r="C18" t="n">
         <v>10</v>
       </c>
       <c r="D18" t="n">
-        <v>0.02054709117463305</v>
+        <v>0.009760555836163753</v>
       </c>
     </row>
     <row r="19">
@@ -686,13 +686,13 @@
         <v>45473</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.01300793123452748</v>
+        <v>-0.01527088325129041</v>
       </c>
       <c r="C19" t="n">
         <v>10</v>
       </c>
       <c r="D19" t="n">
-        <v>0.007271884791036465</v>
+        <v>-0.005659379723768398</v>
       </c>
     </row>
     <row r="20">
@@ -700,13 +700,13 @@
         <v>45504</v>
       </c>
       <c r="B20" t="n">
-        <v>-0.002290435570493921</v>
+        <v>-0.005815950300929873</v>
       </c>
       <c r="C20" t="n">
         <v>10</v>
       </c>
       <c r="D20" t="n">
-        <v>0.004964793436952553</v>
+        <v>-0.01144241535349078</v>
       </c>
     </row>
     <row r="21">
@@ -714,13 +714,13 @@
         <v>45535</v>
       </c>
       <c r="B21" t="n">
-        <v>0.01401574147659729</v>
+        <v>0.01559725598334193</v>
       </c>
       <c r="C21" t="n">
         <v>10</v>
       </c>
       <c r="D21" t="n">
-        <v>0.01905012017484697</v>
+        <v>0.003976370348514946</v>
       </c>
     </row>
     <row r="22">
@@ -728,13 +728,13 @@
         <v>45565</v>
       </c>
       <c r="B22" t="n">
-        <v>0.02231482476539874</v>
+        <v>0.0495629359649389</v>
       </c>
       <c r="C22" t="n">
         <v>10</v>
       </c>
       <c r="D22" t="n">
-        <v>0.0417900450337072</v>
+        <v>0.05373638690241034</v>
       </c>
     </row>
     <row r="23">
@@ -742,13 +742,13 @@
         <v>45596</v>
       </c>
       <c r="B23" t="n">
-        <v>0.0233173285102775</v>
+        <v>0.02602460911316117</v>
       </c>
       <c r="C23" t="n">
         <v>10</v>
       </c>
       <c r="D23" t="n">
-        <v>0.066081805752495</v>
+        <v>0.08115946447986033</v>
       </c>
     </row>
     <row r="24">
@@ -756,13 +756,13 @@
         <v>45626</v>
       </c>
       <c r="B24" t="n">
-        <v>-0.005644976411931952</v>
+        <v>0.001416490980021729</v>
       </c>
       <c r="C24" t="n">
         <v>10</v>
       </c>
       <c r="D24" t="n">
-        <v>0.06006379910583237</v>
+        <v>0.08269091710926135</v>
       </c>
     </row>
     <row r="25">
@@ -770,13 +770,13 @@
         <v>45657</v>
       </c>
       <c r="B25" t="n">
-        <v>0.006359952156123774</v>
+        <v>-0.008400760397969113</v>
       </c>
       <c r="C25" t="n">
         <v>10</v>
       </c>
       <c r="D25" t="n">
-        <v>0.06680575415058421</v>
+        <v>0.07359549012956901</v>
       </c>
     </row>
     <row r="26">
@@ -784,13 +784,13 @@
         <v>45688</v>
       </c>
       <c r="B26" t="n">
-        <v>-0.01428537962067178</v>
+        <v>-0.03586298673230235</v>
       </c>
       <c r="C26" t="n">
         <v>10</v>
       </c>
       <c r="D26" t="n">
-        <v>0.05156602897102602</v>
+        <v>0.03509314931119256</v>
       </c>
     </row>
     <row r="27">
@@ -798,13 +798,13 @@
         <v>45716</v>
       </c>
       <c r="B27" t="n">
-        <v>0.03203715727580259</v>
+        <v>0.04861192443662012</v>
       </c>
       <c r="C27" t="n">
         <v>10</v>
       </c>
       <c r="D27" t="n">
-        <v>0.08525521522706181</v>
+        <v>0.08541101927037142</v>
       </c>
     </row>
     <row r="28">
@@ -812,13 +812,13 @@
         <v>45747</v>
       </c>
       <c r="B28" t="n">
-        <v>0.02805714610413394</v>
+        <v>0.03862605412883276</v>
       </c>
       <c r="C28" t="n">
         <v>10</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1157043793609607</v>
+        <v>0.1273361640527404</v>
       </c>
     </row>
     <row r="29">
@@ -826,13 +826,13 @@
         <v>45777</v>
       </c>
       <c r="B29" t="n">
-        <v>0.009132199460055602</v>
+        <v>0.006104070436585773</v>
       </c>
       <c r="C29" t="n">
         <v>10</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1258932142917424</v>
+        <v>0.1342175034038287</v>
       </c>
     </row>
     <row r="30">
@@ -840,13 +840,13 @@
         <v>45808</v>
       </c>
       <c r="B30" t="n">
-        <v>0.02713230736296136</v>
+        <v>0.02675098929494015</v>
       </c>
       <c r="C30" t="n">
         <v>10</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1564412950397787</v>
+        <v>0.1645589436955184</v>
       </c>
     </row>
     <row r="31">
@@ -854,13 +854,13 @@
         <v>45838</v>
       </c>
       <c r="B31" t="n">
-        <v>0.009625308914002005</v>
+        <v>-4.100550682837115e-06</v>
       </c>
       <c r="C31" t="n">
         <v>10</v>
       </c>
       <c r="D31" t="n">
-        <v>0.167572399745445</v>
+        <v>0.1645541683625467</v>
       </c>
     </row>
     <row r="32">
@@ -868,13 +868,13 @@
         <v>45869</v>
       </c>
       <c r="B32" t="n">
-        <v>0.003476498804306516</v>
+        <v>0.003476473078186004</v>
       </c>
       <c r="C32" t="n">
         <v>10</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1716314637971015</v>
+        <v>0.1686027095769482</v>
       </c>
     </row>
     <row r="33">
@@ -882,13 +882,13 @@
         <v>45900</v>
       </c>
       <c r="B33" t="n">
-        <v>0.0008439908729221957</v>
+        <v>-0.01102386839852076</v>
       </c>
       <c r="C33" t="n">
         <v>10</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1726203100589745</v>
+        <v>0.1557201870964171</v>
       </c>
     </row>
     <row r="34">
@@ -896,13 +896,13 @@
         <v>45930</v>
       </c>
       <c r="B34" t="n">
-        <v>-0.01353785246779336</v>
+        <v>-0.02345834089200296</v>
       </c>
       <c r="C34" t="n">
         <v>10</v>
       </c>
       <c r="D34" t="n">
-        <v>0.156745549300658</v>
+        <v>0.1286089089717399</v>
       </c>
     </row>
     <row r="35">
@@ -910,13 +910,13 @@
         <v>45961</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.013885948088204</v>
+        <v>-0.01811088926475948</v>
       </c>
       <c r="C35" t="n">
         <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>0.140683040651808</v>
+        <v>0.1081687979981318</v>
       </c>
     </row>
     <row r="36">
@@ -924,13 +924,13 @@
         <v>45991</v>
       </c>
       <c r="B36" t="n">
-        <v>0.01562595953869194</v>
+        <v>0.0135162932890513</v>
       </c>
       <c r="C36" t="n">
         <v>10</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1585073076915051</v>
+        <v>0.1231471324856501</v>
       </c>
     </row>
   </sheetData>
@@ -999,28 +999,28 @@
         <v>44957</v>
       </c>
       <c r="B2" t="n">
-        <v>0.01327584140617164</v>
+        <v>-0.0143223005375106</v>
       </c>
       <c r="C2" t="n">
         <v>0.01283122455642394</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02610706596259558</v>
+        <v>-0.001491075981086665</v>
       </c>
       <c r="E2" t="n">
         <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01327584140617155</v>
+        <v>-0.0143223005375106</v>
       </c>
       <c r="G2" t="n">
-        <v>0.02610706596259549</v>
+        <v>-0.001491075981086665</v>
       </c>
       <c r="H2" t="n">
         <v>0.01283122455642394</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01327584140617155</v>
+        <v>-0.0143223005375106</v>
       </c>
     </row>
     <row r="3">
@@ -1028,28 +1028,28 @@
         <v>44985</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.007811532004062349</v>
+        <v>0.01759315770546228</v>
       </c>
       <c r="C3" t="n">
         <v>-0.001347254968002698</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.009158786972065047</v>
+        <v>0.01624590273745958</v>
       </c>
       <c r="E3" t="n">
         <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>0.005360604742083996</v>
+        <v>0.003018882675890122</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01670916993491334</v>
+        <v>0.01473060288100991</v>
       </c>
       <c r="H3" t="n">
         <v>0.01146668265739215</v>
       </c>
       <c r="I3" t="n">
-        <v>0.005242487277521191</v>
+        <v>0.003263920223617767</v>
       </c>
     </row>
     <row r="4">
@@ -1057,28 +1057,28 @@
         <v>45016</v>
       </c>
       <c r="B4" t="n">
-        <v>9.650945197502148e-06</v>
+        <v>9.642576345149367e-06</v>
       </c>
       <c r="C4" t="n">
         <v>0.02105905705452504</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02106870799972255</v>
+        <v>0.02106869963087019</v>
       </c>
       <c r="E4" t="n">
         <v>10</v>
       </c>
       <c r="F4" t="n">
-        <v>0.005370307422184029</v>
+        <v>0.00302855436204208</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03812991855691217</v>
+        <v>0.03610965715936176</v>
       </c>
       <c r="H4" t="n">
         <v>0.03276721723622544</v>
       </c>
       <c r="I4" t="n">
-        <v>0.005362701320686725</v>
+        <v>0.00334243992313632</v>
       </c>
     </row>
     <row r="5">
@@ -1086,28 +1086,28 @@
         <v>45046</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.03159173821935352</v>
+        <v>-0.02840761119052029</v>
       </c>
       <c r="C5" t="n">
         <v>-0.01568767273643767</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.04727941095579119</v>
+        <v>-0.04409528392695796</v>
       </c>
       <c r="E5" t="n">
         <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.02639108814340863</v>
+        <v>-0.02546509082326442</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.01095225248804221</v>
+        <v>-0.00957789235254336</v>
       </c>
       <c r="H5" t="n">
         <v>0.01656550311930216</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.02751775560734437</v>
+        <v>-0.02614339547184552</v>
       </c>
     </row>
     <row r="6">
@@ -1115,28 +1115,28 @@
         <v>45077</v>
       </c>
       <c r="B6" t="n">
-        <v>0.05360188891873661</v>
+        <v>0.0138504850058213</v>
       </c>
       <c r="C6" t="n">
         <v>0.03353077581524766</v>
       </c>
       <c r="D6" t="n">
-        <v>0.08713266473398426</v>
+        <v>0.04738126082106896</v>
       </c>
       <c r="E6" t="n">
         <v>10</v>
       </c>
       <c r="F6" t="n">
-        <v>0.02579618860022048</v>
+        <v>-0.01196730967606274</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0752261133018195</v>
+        <v>0.0373495558528536</v>
       </c>
       <c r="H6" t="n">
         <v>0.05065173310590998</v>
       </c>
       <c r="I6" t="n">
-        <v>0.02457438019590952</v>
+        <v>-0.01330217725305638</v>
       </c>
     </row>
     <row r="7">
@@ -1144,28 +1144,28 @@
         <v>45107</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.0005059612217292618</v>
+        <v>-0.006580249463349672</v>
       </c>
       <c r="C7" t="n">
         <v>-0.02553356550597963</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.02603952672770889</v>
+        <v>-0.0321138149693293</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>0.02527717550739106</v>
+        <v>-0.01846881125633881</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04722773418616621</v>
+        <v>0.004036304157679194</v>
       </c>
       <c r="H7" t="n">
         <v>0.02382484825467923</v>
       </c>
       <c r="I7" t="n">
-        <v>0.02340288593148698</v>
+        <v>-0.01978854409700004</v>
       </c>
     </row>
     <row r="8">
@@ -1173,28 +1173,28 @@
         <v>45138</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.01441718927685273</v>
+        <v>-0.01107544251413588</v>
       </c>
       <c r="C8" t="n">
         <v>-0.02940128211469095</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.04381847139154368</v>
+        <v>-0.04047672462882683</v>
       </c>
       <c r="E8" t="n">
         <v>10</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01049556040686395</v>
+        <v>-0.02933970351310067</v>
       </c>
       <c r="G8" t="n">
-        <v>0.001339815675298617</v>
+        <v>-0.03660379684305615</v>
       </c>
       <c r="H8" t="n">
         <v>-0.006276914944887246</v>
       </c>
       <c r="I8" t="n">
-        <v>0.007616730620185863</v>
+        <v>-0.0303268818981689</v>
       </c>
     </row>
     <row r="9">
@@ -1202,28 +1202,28 @@
         <v>45169</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.01777729036170989</v>
+        <v>-0.01777727761230753</v>
       </c>
       <c r="C9" t="n">
         <v>-0.01338832086689734</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.03116561122860723</v>
+        <v>-0.03116559847920487</v>
       </c>
       <c r="E9" t="n">
         <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.007468312579707703</v>
+        <v>-0.04659540107099303</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.0298675517277629</v>
+        <v>-0.06662861608703596</v>
       </c>
       <c r="H9" t="n">
         <v>-0.01958119846044826</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.01028635326731464</v>
+        <v>-0.04704741762658771</v>
       </c>
     </row>
     <row r="10">
@@ -1231,28 +1231,28 @@
         <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>0.004491610576988268</v>
+        <v>0.001572329559243646</v>
       </c>
       <c r="C10" t="n">
         <v>-0.03697532882683852</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.03248371824985025</v>
+        <v>-0.03540299926759487</v>
       </c>
       <c r="E10" t="n">
         <v>10</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.003010246754494683</v>
+        <v>-0.04509633483817821</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.06138106084247574</v>
+        <v>-0.09967276250810064</v>
       </c>
       <c r="H10" t="n">
         <v>-0.05583250603538814</v>
       </c>
       <c r="I10" t="n">
-        <v>-0.005548554807087602</v>
+        <v>-0.0438402564727125</v>
       </c>
     </row>
     <row r="11">
@@ -1260,28 +1260,28 @@
         <v>45230</v>
       </c>
       <c r="B11" t="n">
-        <v>0.03907173562954228</v>
+        <v>0.03907176541251828</v>
       </c>
       <c r="C11" t="n">
         <v>0.07547484038691965</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1145465760164619</v>
+        <v>0.1145466057994379</v>
       </c>
       <c r="E11" t="n">
         <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>0.03594387330967619</v>
+        <v>-0.00778656284142154</v>
       </c>
       <c r="G11" t="n">
-        <v>0.04613452482222247</v>
+        <v>0.003456666655381024</v>
       </c>
       <c r="H11" t="n">
         <v>0.01542838487010889</v>
       </c>
       <c r="I11" t="n">
-        <v>0.03070613995211358</v>
+        <v>-0.01197171821472787</v>
       </c>
     </row>
     <row r="12">
@@ -1289,28 +1289,28 @@
         <v>45260</v>
       </c>
       <c r="B12" t="n">
-        <v>0.025319759910151</v>
+        <v>0.01324342021713043</v>
       </c>
       <c r="C12" t="n">
         <v>0.0742275175532876</v>
       </c>
       <c r="D12" t="n">
-        <v>0.09954727746343861</v>
+        <v>0.08747093777041803</v>
       </c>
       <c r="E12" t="n">
         <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>0.06217372346226901</v>
+        <v>0.005353736651952934</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1502743686287829</v>
+        <v>0.09122996229970481</v>
       </c>
       <c r="H12" t="n">
         <v>0.09080111313216133</v>
       </c>
       <c r="I12" t="n">
-        <v>0.05947325549662152</v>
+        <v>0.000428849167543488</v>
       </c>
     </row>
     <row r="13">
@@ -1318,28 +1318,28 @@
         <v>45291</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.02513223480897647</v>
+        <v>-0.03629742036736827</v>
       </c>
       <c r="C13" t="n">
         <v>-0.01733397781348567</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.04246621262246213</v>
+        <v>-0.05363139818085394</v>
       </c>
       <c r="E13" t="n">
         <v>10</v>
       </c>
       <c r="F13" t="n">
-        <v>0.03547892403629049</v>
+        <v>-0.03113801054520748</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1014265727164245</v>
+        <v>0.03270577368473115</v>
       </c>
       <c r="H13" t="n">
         <v>0.071893190838203</v>
       </c>
       <c r="I13" t="n">
-        <v>0.02953338187822152</v>
+        <v>-0.03918741715347185</v>
       </c>
     </row>
     <row r="14">
@@ -1347,28 +1347,28 @@
         <v>45322</v>
       </c>
       <c r="B14" t="n">
-        <v>-0.0308767377645388</v>
+        <v>-0.0285878551922281</v>
       </c>
       <c r="C14" t="n">
         <v>0.04082574766638825</v>
       </c>
       <c r="D14" t="n">
-        <v>0.009949009901849448</v>
+        <v>0.01223789247416015</v>
       </c>
       <c r="E14" t="n">
         <v>10</v>
       </c>
       <c r="F14" t="n">
-        <v>0.003506712838115211</v>
+        <v>-0.0588356968009951</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1123846765945404</v>
+        <v>0.04534391590052933</v>
       </c>
       <c r="H14" t="n">
         <v>0.1156540317726833</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.003269355178142863</v>
+        <v>-0.07031011587215397</v>
       </c>
     </row>
     <row r="15">
@@ -1376,28 +1376,28 @@
         <v>45351</v>
       </c>
       <c r="B15" t="n">
-        <v>0.05501209632906345</v>
+        <v>0.05362457887198531</v>
       </c>
       <c r="C15" t="n">
         <v>0.02668774155917708</v>
       </c>
       <c r="D15" t="n">
-        <v>0.08169983788824053</v>
+        <v>0.08031232043116239</v>
       </c>
       <c r="E15" t="n">
         <v>10</v>
       </c>
       <c r="F15" t="n">
-        <v>0.05871172079162745</v>
+        <v>-0.008366157392602935</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2032663243416772</v>
+        <v>0.1292979114350987</v>
       </c>
       <c r="H15" t="n">
         <v>0.1454283182420866</v>
       </c>
       <c r="I15" t="n">
-        <v>0.05783800609959067</v>
+        <v>-0.01613040680698785</v>
       </c>
     </row>
     <row r="16">
@@ -1405,28 +1405,28 @@
         <v>45382</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.04502231949049337</v>
+        <v>-0.005100952935510233</v>
       </c>
       <c r="C16" t="n">
         <v>0.01514130038350592</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.02988101910698745</v>
+        <v>0.01004034744799568</v>
       </c>
       <c r="E16" t="n">
         <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>0.01104606344981685</v>
+        <v>-0.0134244349530025</v>
       </c>
       <c r="G16" t="n">
-        <v>0.1673115003132291</v>
+        <v>0.1406364548382031</v>
       </c>
       <c r="H16" t="n">
         <v>0.162771592476364</v>
       </c>
       <c r="I16" t="n">
-        <v>0.004539907836865087</v>
+        <v>-0.02213513763816088</v>
       </c>
     </row>
     <row r="17">
@@ -1434,28 +1434,28 @@
         <v>45412</v>
       </c>
       <c r="B17" t="n">
-        <v>0.01505408354698202</v>
+        <v>0.01418645548354154</v>
       </c>
       <c r="C17" t="n">
         <v>0.01865912890575827</v>
       </c>
       <c r="D17" t="n">
-        <v>0.03371321245274029</v>
+        <v>0.03284558438929981</v>
       </c>
       <c r="E17" t="n">
         <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>0.02626643535883777</v>
+        <v>0.0005715753816866176</v>
       </c>
       <c r="G17" t="n">
-        <v>0.2066653209218161</v>
+        <v>0.178101325773103</v>
       </c>
       <c r="H17" t="n">
         <v>0.1844678975083343</v>
       </c>
       <c r="I17" t="n">
-        <v>0.02219742341348185</v>
+        <v>-0.006366571735231252</v>
       </c>
     </row>
     <row r="18">
@@ -1463,28 +1463,28 @@
         <v>45443</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.00557296232942169</v>
+        <v>0.009183731259777062</v>
       </c>
       <c r="C18" t="n">
         <v>-0.01330599638453256</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.01887895871395425</v>
+        <v>-0.004122265124755498</v>
       </c>
       <c r="E18" t="n">
         <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>0.02054709117463305</v>
+        <v>0.009760555836163753</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1838847361465727</v>
+        <v>0.1732448797644404</v>
       </c>
       <c r="H18" t="n">
         <v>0.1687073719464935</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0151773642000792</v>
+        <v>0.004537507817946818</v>
       </c>
     </row>
     <row r="19">
@@ -1492,28 +1492,28 @@
         <v>45473</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.01300793123452748</v>
+        <v>-0.01527088325129041</v>
       </c>
       <c r="C19" t="n">
         <v>0.01552088100993609</v>
       </c>
       <c r="D19" t="n">
-        <v>0.002512949775408613</v>
+        <v>0.0002499977586456811</v>
       </c>
       <c r="E19" t="n">
         <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>0.007271884791036465</v>
+        <v>-0.005659379723768398</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1868597790283819</v>
+        <v>0.173538188354724</v>
       </c>
       <c r="H19" t="n">
         <v>0.1868467400019103</v>
       </c>
       <c r="I19" t="n">
-        <v>1.303902647165067e-05</v>
+        <v>-0.01330855164718625</v>
       </c>
     </row>
     <row r="20">
@@ -1521,28 +1521,28 @@
         <v>45504</v>
       </c>
       <c r="B20" t="n">
-        <v>-0.002290435570493921</v>
+        <v>-0.005815950300929873</v>
       </c>
       <c r="C20" t="n">
         <v>-0.005123965457489166</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.007414401027983086</v>
+        <v>-0.01093991575841904</v>
       </c>
       <c r="E20" t="n">
         <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>0.004964793436952553</v>
+        <v>-0.01144241535349078</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1780599246626822</v>
+        <v>0.1606997794348357</v>
       </c>
       <c r="H20" t="n">
         <v>0.1807653783028069</v>
       </c>
       <c r="I20" t="n">
-        <v>-0.002705453640124755</v>
+        <v>-0.02006559886797121</v>
       </c>
     </row>
     <row r="21">
@@ -1550,28 +1550,28 @@
         <v>45535</v>
       </c>
       <c r="B21" t="n">
-        <v>0.01401574147659729</v>
+        <v>0.01559725598334193</v>
       </c>
       <c r="C21" t="n">
         <v>0.01174131378272203</v>
       </c>
       <c r="D21" t="n">
-        <v>0.02575705525931932</v>
+        <v>0.02733856976606396</v>
       </c>
       <c r="E21" t="n">
         <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>0.01905012017484697</v>
+        <v>0.003976370348514946</v>
       </c>
       <c r="G21" t="n">
-        <v>0.2084032792410084</v>
+        <v>0.1924316513323701</v>
       </c>
       <c r="H21" t="n">
         <v>0.1946291151132347</v>
       </c>
       <c r="I21" t="n">
-        <v>0.01377416412777377</v>
+        <v>-0.002197463780864606</v>
       </c>
     </row>
     <row r="22">
@@ -1579,28 +1579,28 @@
         <v>45565</v>
       </c>
       <c r="B22" t="n">
-        <v>0.02231482476539874</v>
+        <v>0.0495629359649389</v>
       </c>
       <c r="C22" t="n">
         <v>-0.03199388951261672</v>
       </c>
       <c r="D22" t="n">
-        <v>-0.00967906474721798</v>
+        <v>0.01756904645232218</v>
       </c>
       <c r="E22" t="n">
         <v>10</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0417900450337072</v>
+        <v>0.05373638690241034</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1967070656604841</v>
+        <v>0.2133815384058477</v>
       </c>
       <c r="H22" t="n">
         <v>0.1564082831957467</v>
       </c>
       <c r="I22" t="n">
-        <v>0.04029878246473739</v>
+        <v>0.05697325521010099</v>
       </c>
     </row>
     <row r="23">
@@ -1608,28 +1608,28 @@
         <v>45596</v>
       </c>
       <c r="B23" t="n">
-        <v>0.0233173285102775</v>
+        <v>0.02602460911316117</v>
       </c>
       <c r="C23" t="n">
         <v>-0.01123336339946446</v>
       </c>
       <c r="D23" t="n">
-        <v>0.01208396511081304</v>
+        <v>0.01479124571369671</v>
       </c>
       <c r="E23" t="n">
         <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>0.066081805752495</v>
+        <v>0.08115946447986033</v>
       </c>
       <c r="G23" t="n">
-        <v>0.2111680320897888</v>
+        <v>0.231328962884872</v>
       </c>
       <c r="H23" t="n">
         <v>0.1434179287124582</v>
       </c>
       <c r="I23" t="n">
-        <v>0.06775010337733067</v>
+        <v>0.08791103417241386</v>
       </c>
     </row>
     <row r="24">
@@ -1637,28 +1637,28 @@
         <v>45626</v>
       </c>
       <c r="B24" t="n">
-        <v>-0.005644976411931952</v>
+        <v>0.001416490980021729</v>
       </c>
       <c r="C24" t="n">
         <v>-0.01222426925829856</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.01786924567023051</v>
+        <v>-0.01080777827827683</v>
       </c>
       <c r="E24" t="n">
         <v>10</v>
       </c>
       <c r="F24" t="n">
-        <v>0.06006379910583237</v>
+        <v>0.08269091710926135</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1895253729764468</v>
+        <v>0.2180210324663918</v>
       </c>
       <c r="H24" t="n">
         <v>0.129440480077111</v>
       </c>
       <c r="I24" t="n">
-        <v>0.06008489289933583</v>
+        <v>0.08858055238928086</v>
       </c>
     </row>
     <row r="25">
@@ -1666,28 +1666,28 @@
         <v>45657</v>
       </c>
       <c r="B25" t="n">
-        <v>0.006359952156123774</v>
+        <v>-0.008400760397969113</v>
       </c>
       <c r="C25" t="n">
         <v>0.0754775898989859</v>
       </c>
       <c r="D25" t="n">
-        <v>0.08183754205510967</v>
+        <v>0.06707682950101679</v>
       </c>
       <c r="E25" t="n">
         <v>10</v>
       </c>
       <c r="F25" t="n">
-        <v>0.06680575415058421</v>
+        <v>0.07359549012956901</v>
       </c>
       <c r="G25" t="n">
-        <v>0.2868732057130268</v>
+        <v>0.2997220215897924</v>
       </c>
       <c r="H25" t="n">
         <v>0.2146879254476848</v>
       </c>
       <c r="I25" t="n">
-        <v>0.07218528026534199</v>
+        <v>0.08503409614210766</v>
       </c>
     </row>
     <row r="26">
@@ -1695,28 +1695,28 @@
         <v>45688</v>
       </c>
       <c r="B26" t="n">
-        <v>-0.01428537962067178</v>
+        <v>-0.03586298673230235</v>
       </c>
       <c r="C26" t="n">
         <v>0.02028050930417358</v>
       </c>
       <c r="D26" t="n">
-        <v>0.005995129683501799</v>
+        <v>-0.01558247742812877</v>
       </c>
       <c r="E26" t="n">
         <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>0.05156602897102602</v>
+        <v>0.03509314931119256</v>
       </c>
       <c r="G26" t="n">
-        <v>0.2945881774674999</v>
+        <v>0.2794691325255276</v>
       </c>
       <c r="H26" t="n">
         <v>0.2393224152213937</v>
       </c>
       <c r="I26" t="n">
-        <v>0.05526576224610613</v>
+        <v>0.04014671730413388</v>
       </c>
     </row>
     <row r="27">
@@ -1724,28 +1724,28 @@
         <v>45716</v>
       </c>
       <c r="B27" t="n">
-        <v>0.03203715727580259</v>
+        <v>0.04861192443662012</v>
       </c>
       <c r="C27" t="n">
         <v>-0.08464781323129844</v>
       </c>
       <c r="D27" t="n">
-        <v>-0.05261065595549586</v>
+        <v>-0.03603588879467833</v>
       </c>
       <c r="E27" t="n">
         <v>10</v>
       </c>
       <c r="F27" t="n">
-        <v>0.08525521522706181</v>
+        <v>0.08541101927037142</v>
       </c>
       <c r="G27" t="n">
-        <v>0.2264790442587048</v>
+        <v>0.2333623251496142</v>
       </c>
       <c r="H27" t="n">
         <v>0.1344164828843715</v>
       </c>
       <c r="I27" t="n">
-        <v>0.09206256137433333</v>
+        <v>0.09894584226524272</v>
       </c>
     </row>
     <row r="28">
@@ -1753,28 +1753,28 @@
         <v>45747</v>
       </c>
       <c r="B28" t="n">
-        <v>0.02805714610413394</v>
+        <v>0.03862605412883276</v>
       </c>
       <c r="C28" t="n">
         <v>-0.02405715924653007</v>
       </c>
       <c r="D28" t="n">
-        <v>0.003999986857603867</v>
+        <v>0.0145688948823027</v>
       </c>
       <c r="E28" t="n">
         <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>0.1157043793609607</v>
+        <v>0.1273361640527404</v>
       </c>
       <c r="G28" t="n">
-        <v>0.2313849443168663</v>
+        <v>0.2513310512165112</v>
       </c>
       <c r="H28" t="n">
         <v>0.1071256449037337</v>
       </c>
       <c r="I28" t="n">
-        <v>0.1242592994131326</v>
+        <v>0.1442054063127776</v>
       </c>
     </row>
     <row r="29">
@@ -1782,28 +1782,28 @@
         <v>45777</v>
       </c>
       <c r="B29" t="n">
-        <v>0.009132199460055602</v>
+        <v>0.006104070436585773</v>
       </c>
       <c r="C29" t="n">
         <v>0.02546362003267832</v>
       </c>
       <c r="D29" t="n">
-        <v>0.03459581949273392</v>
+        <v>0.0315676904692641</v>
       </c>
       <c r="E29" t="n">
         <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1258932142917424</v>
+        <v>0.1342175034038287</v>
       </c>
       <c r="G29" t="n">
-        <v>0.2739857155765226</v>
+        <v>0.2908326825158929</v>
       </c>
       <c r="H29" t="n">
         <v>0.1353170716539962</v>
       </c>
       <c r="I29" t="n">
-        <v>0.1386686439225264</v>
+        <v>0.1555156108618967</v>
       </c>
     </row>
     <row r="30">
@@ -1811,28 +1811,28 @@
         <v>45808</v>
       </c>
       <c r="B30" t="n">
-        <v>0.02713230736296136</v>
+        <v>0.02675098929494015</v>
       </c>
       <c r="C30" t="n">
         <v>-0.0010176275311089</v>
       </c>
       <c r="D30" t="n">
-        <v>0.02611467983185246</v>
+        <v>0.02573336176383125</v>
       </c>
       <c r="E30" t="n">
         <v>10</v>
       </c>
       <c r="F30" t="n">
-        <v>0.1564412950397787</v>
+        <v>0.1645589436955184</v>
       </c>
       <c r="G30" t="n">
-        <v>0.3072554446491571</v>
+        <v>0.3240501469116512</v>
       </c>
       <c r="H30" t="n">
         <v>0.1341617417453431</v>
       </c>
       <c r="I30" t="n">
-        <v>0.173093702903814</v>
+        <v>0.1898884051663081</v>
       </c>
     </row>
     <row r="31">
@@ -1840,28 +1840,28 @@
         <v>45838</v>
       </c>
       <c r="B31" t="n">
-        <v>0.009625308914002005</v>
+        <v>-4.100550682837115e-06</v>
       </c>
       <c r="C31" t="n">
         <v>0.03471026622343087</v>
       </c>
       <c r="D31" t="n">
-        <v>0.04433557513743288</v>
+        <v>0.03470616567274803</v>
       </c>
       <c r="E31" t="n">
         <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>0.167572399745445</v>
+        <v>0.1645541683625467</v>
       </c>
       <c r="G31" t="n">
-        <v>0.3652133666392179</v>
+        <v>0.3700028506693935</v>
       </c>
       <c r="H31" t="n">
         <v>0.1735287977417541</v>
       </c>
       <c r="I31" t="n">
-        <v>0.1916845688974638</v>
+        <v>0.1964740529276394</v>
       </c>
     </row>
     <row r="32">
@@ -1869,28 +1869,28 @@
         <v>45869</v>
       </c>
       <c r="B32" t="n">
-        <v>0.003476498804306516</v>
+        <v>0.003476473078186004</v>
       </c>
       <c r="C32" t="n">
         <v>0.01769341736780827</v>
       </c>
       <c r="D32" t="n">
-        <v>0.02116991617211479</v>
+        <v>0.02116989044599428</v>
       </c>
       <c r="E32" t="n">
         <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>0.1716314637971015</v>
+        <v>0.1686027095769482</v>
       </c>
       <c r="G32" t="n">
-        <v>0.3941148191680208</v>
+        <v>0.3990056609287644</v>
       </c>
       <c r="H32" t="n">
         <v>0.1942925325533413</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1998222866146795</v>
+        <v>0.2047131283754231</v>
       </c>
     </row>
     <row r="33">
@@ -1898,28 +1898,28 @@
         <v>45900</v>
       </c>
       <c r="B33" t="n">
-        <v>0.0008439908729221957</v>
+        <v>-0.01102386839852076</v>
       </c>
       <c r="C33" t="n">
         <v>0.01412960290443377</v>
       </c>
       <c r="D33" t="n">
-        <v>0.01497359377735596</v>
+        <v>0.003105734505913005</v>
       </c>
       <c r="E33" t="n">
         <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>0.1726203100589745</v>
+        <v>0.1557201870964171</v>
       </c>
       <c r="G33" t="n">
-        <v>0.414989728149235</v>
+        <v>0.4033506010838788</v>
       </c>
       <c r="H33" t="n">
         <v>0.2111674117900506</v>
       </c>
       <c r="I33" t="n">
-        <v>0.2038223163591844</v>
+        <v>0.1921831892938282</v>
       </c>
     </row>
     <row r="34">
@@ -1927,28 +1927,28 @@
         <v>45930</v>
       </c>
       <c r="B34" t="n">
-        <v>-0.01353785246779336</v>
+        <v>-0.02345834089200296</v>
       </c>
       <c r="C34" t="n">
         <v>0.0391580357590644</v>
       </c>
       <c r="D34" t="n">
-        <v>0.02562018329127104</v>
+        <v>0.01569969486706144</v>
       </c>
       <c r="E34" t="n">
         <v>10</v>
       </c>
       <c r="F34" t="n">
-        <v>0.156745549300658</v>
+        <v>0.1286089089717399</v>
       </c>
       <c r="G34" t="n">
-        <v>0.4512420243396842</v>
+        <v>0.4253827773124028</v>
       </c>
       <c r="H34" t="n">
         <v>0.2585943486111388</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1926476757285454</v>
+        <v>0.166788428701264</v>
       </c>
     </row>
     <row r="35">
@@ -1956,28 +1956,28 @@
         <v>45961</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.013885948088204</v>
+        <v>-0.01811088926475948</v>
       </c>
       <c r="C35" t="n">
         <v>0.00748081930001443</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.006405128788189574</v>
+        <v>-0.01063006996474505</v>
       </c>
       <c r="E35" t="n">
         <v>10</v>
       </c>
       <c r="F35" t="n">
-        <v>0.140683040651808</v>
+        <v>0.1081687979981318</v>
       </c>
       <c r="G35" t="n">
-        <v>0.4419466322709555</v>
+        <v>0.4102308586630294</v>
       </c>
       <c r="H35" t="n">
         <v>0.2680096655051181</v>
       </c>
       <c r="I35" t="n">
-        <v>0.1739369667658375</v>
+        <v>0.1422211931579114</v>
       </c>
     </row>
     <row r="36">
@@ -1985,28 +1985,28 @@
         <v>45991</v>
       </c>
       <c r="B36" t="n">
-        <v>0.01562595953869194</v>
+        <v>0.0135162932890513</v>
       </c>
       <c r="C36" t="n">
         <v>0.0341491408921466</v>
       </c>
       <c r="D36" t="n">
-        <v>0.04977510043083853</v>
+        <v>0.0476654341811979</v>
       </c>
       <c r="E36" t="n">
         <v>10</v>
       </c>
       <c r="F36" t="n">
-        <v>0.1585073076915051</v>
+        <v>0.1231471324856501</v>
       </c>
       <c r="G36" t="n">
-        <v>0.5137196707081517</v>
+        <v>0.4774501248369263</v>
       </c>
       <c r="H36" t="n">
         <v>0.311311106225056</v>
       </c>
       <c r="I36" t="n">
-        <v>0.2024085644830957</v>
+        <v>0.1661390186118703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>